<commit_message>
Staff schedule page with team logins and a message board; employee emails in the admin table
- team/: employees create their own login (only emails on the staff list can), see their shifts,
  who's working each day (first name + last initial and position only) and a live message board
- Admin Employees tab: Email (login) and Login status columns, team page link, import reads Email
- supabase/team.sql: email column, staff-list-only sign-ups, team_schedule() that returns published
  shifts without contact details, board_posts with author names set by the database
- Home tile for the staff page; employees who open the manager site are pointed to it

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019NsoWEujssTsfRwL36NJVa
</commit_message>
<xml_diff>
--- a/templates/eden-employees.xlsx
+++ b/templates/eden-employees.xlsx
@@ -85,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -95,7 +95,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -463,13 +462,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D81"/>
+  <dimension ref="A1:E81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -482,7 +482,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fill in one row per employee in the yellow cells (name and mobile number are the important ones). Any phone format works, e.g. 315-555-0123.</t>
+          <t>Fill in one row per employee in the yellow cells. Any phone format works, e.g. 315-555-0123. The email is what they use to create their login for the staff schedule page.</t>
         </is>
       </c>
     </row>
@@ -506,10 +506,15 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
+          <t>Email (staff page login)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
           <t>Position</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Notes (not imported)</t>
         </is>
@@ -521,479 +526,559 @@
           <t>Example: Jane Smith</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>(315) 555-0123</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
+          <t>jane@example.com</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
           <t>Server</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>Example row, leave as is or delete</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="n"/>
-      <c r="B7" s="7" t="n"/>
+      <c r="A7" s="5" t="n"/>
+      <c r="B7" s="6" t="n"/>
       <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="n"/>
-      <c r="B8" s="7" t="n"/>
+      <c r="A8" s="5" t="n"/>
+      <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="5" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="n"/>
-      <c r="B9" s="7" t="n"/>
+      <c r="A9" s="5" t="n"/>
+      <c r="B9" s="6" t="n"/>
       <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="n"/>
-      <c r="B10" s="7" t="n"/>
+      <c r="A10" s="5" t="n"/>
+      <c r="B10" s="6" t="n"/>
       <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="n"/>
-      <c r="B11" s="7" t="n"/>
+      <c r="A11" s="5" t="n"/>
+      <c r="B11" s="6" t="n"/>
       <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="5" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="n"/>
-      <c r="B12" s="7" t="n"/>
+      <c r="A12" s="5" t="n"/>
+      <c r="B12" s="6" t="n"/>
       <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="n"/>
-      <c r="B13" s="7" t="n"/>
+      <c r="A13" s="5" t="n"/>
+      <c r="B13" s="6" t="n"/>
       <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="n"/>
-      <c r="B14" s="7" t="n"/>
+      <c r="A14" s="5" t="n"/>
+      <c r="B14" s="6" t="n"/>
       <c r="C14" s="6" t="n"/>
-      <c r="D14" s="6" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="n"/>
-      <c r="B15" s="7" t="n"/>
+      <c r="A15" s="5" t="n"/>
+      <c r="B15" s="6" t="n"/>
       <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="n"/>
-      <c r="B16" s="7" t="n"/>
+      <c r="A16" s="5" t="n"/>
+      <c r="B16" s="6" t="n"/>
       <c r="C16" s="6" t="n"/>
-      <c r="D16" s="6" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="n"/>
-      <c r="B17" s="7" t="n"/>
+      <c r="A17" s="5" t="n"/>
+      <c r="B17" s="6" t="n"/>
       <c r="C17" s="6" t="n"/>
-      <c r="D17" s="6" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="n"/>
-      <c r="B18" s="7" t="n"/>
+      <c r="A18" s="5" t="n"/>
+      <c r="B18" s="6" t="n"/>
       <c r="C18" s="6" t="n"/>
-      <c r="D18" s="6" t="n"/>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="5" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="7" t="n"/>
+      <c r="A19" s="5" t="n"/>
+      <c r="B19" s="6" t="n"/>
       <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6" t="n"/>
+      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="5" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="n"/>
-      <c r="B20" s="7" t="n"/>
+      <c r="A20" s="5" t="n"/>
+      <c r="B20" s="6" t="n"/>
       <c r="C20" s="6" t="n"/>
-      <c r="D20" s="6" t="n"/>
+      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="5" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="n"/>
-      <c r="B21" s="7" t="n"/>
+      <c r="A21" s="5" t="n"/>
+      <c r="B21" s="6" t="n"/>
       <c r="C21" s="6" t="n"/>
-      <c r="D21" s="6" t="n"/>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="5" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="n"/>
-      <c r="B22" s="7" t="n"/>
+      <c r="A22" s="5" t="n"/>
+      <c r="B22" s="6" t="n"/>
       <c r="C22" s="6" t="n"/>
-      <c r="D22" s="6" t="n"/>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="n"/>
-      <c r="B23" s="7" t="n"/>
+      <c r="A23" s="5" t="n"/>
+      <c r="B23" s="6" t="n"/>
       <c r="C23" s="6" t="n"/>
-      <c r="D23" s="6" t="n"/>
+      <c r="D23" s="5" t="n"/>
+      <c r="E23" s="5" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="n"/>
-      <c r="B24" s="7" t="n"/>
+      <c r="A24" s="5" t="n"/>
+      <c r="B24" s="6" t="n"/>
       <c r="C24" s="6" t="n"/>
-      <c r="D24" s="6" t="n"/>
+      <c r="D24" s="5" t="n"/>
+      <c r="E24" s="5" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="n"/>
-      <c r="B25" s="7" t="n"/>
+      <c r="A25" s="5" t="n"/>
+      <c r="B25" s="6" t="n"/>
       <c r="C25" s="6" t="n"/>
-      <c r="D25" s="6" t="n"/>
+      <c r="D25" s="5" t="n"/>
+      <c r="E25" s="5" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="n"/>
-      <c r="B26" s="7" t="n"/>
+      <c r="A26" s="5" t="n"/>
+      <c r="B26" s="6" t="n"/>
       <c r="C26" s="6" t="n"/>
-      <c r="D26" s="6" t="n"/>
+      <c r="D26" s="5" t="n"/>
+      <c r="E26" s="5" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="n"/>
-      <c r="B27" s="7" t="n"/>
+      <c r="A27" s="5" t="n"/>
+      <c r="B27" s="6" t="n"/>
       <c r="C27" s="6" t="n"/>
-      <c r="D27" s="6" t="n"/>
+      <c r="D27" s="5" t="n"/>
+      <c r="E27" s="5" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="n"/>
-      <c r="B28" s="7" t="n"/>
+      <c r="A28" s="5" t="n"/>
+      <c r="B28" s="6" t="n"/>
       <c r="C28" s="6" t="n"/>
-      <c r="D28" s="6" t="n"/>
+      <c r="D28" s="5" t="n"/>
+      <c r="E28" s="5" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="n"/>
-      <c r="B29" s="7" t="n"/>
+      <c r="A29" s="5" t="n"/>
+      <c r="B29" s="6" t="n"/>
       <c r="C29" s="6" t="n"/>
-      <c r="D29" s="6" t="n"/>
+      <c r="D29" s="5" t="n"/>
+      <c r="E29" s="5" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="n"/>
-      <c r="B30" s="7" t="n"/>
+      <c r="A30" s="5" t="n"/>
+      <c r="B30" s="6" t="n"/>
       <c r="C30" s="6" t="n"/>
-      <c r="D30" s="6" t="n"/>
+      <c r="D30" s="5" t="n"/>
+      <c r="E30" s="5" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="n"/>
-      <c r="B31" s="7" t="n"/>
+      <c r="A31" s="5" t="n"/>
+      <c r="B31" s="6" t="n"/>
       <c r="C31" s="6" t="n"/>
-      <c r="D31" s="6" t="n"/>
+      <c r="D31" s="5" t="n"/>
+      <c r="E31" s="5" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="n"/>
-      <c r="B32" s="7" t="n"/>
+      <c r="A32" s="5" t="n"/>
+      <c r="B32" s="6" t="n"/>
       <c r="C32" s="6" t="n"/>
-      <c r="D32" s="6" t="n"/>
+      <c r="D32" s="5" t="n"/>
+      <c r="E32" s="5" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="n"/>
-      <c r="B33" s="7" t="n"/>
+      <c r="A33" s="5" t="n"/>
+      <c r="B33" s="6" t="n"/>
       <c r="C33" s="6" t="n"/>
-      <c r="D33" s="6" t="n"/>
+      <c r="D33" s="5" t="n"/>
+      <c r="E33" s="5" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="n"/>
-      <c r="B34" s="7" t="n"/>
+      <c r="A34" s="5" t="n"/>
+      <c r="B34" s="6" t="n"/>
       <c r="C34" s="6" t="n"/>
-      <c r="D34" s="6" t="n"/>
+      <c r="D34" s="5" t="n"/>
+      <c r="E34" s="5" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="n"/>
-      <c r="B35" s="7" t="n"/>
+      <c r="A35" s="5" t="n"/>
+      <c r="B35" s="6" t="n"/>
       <c r="C35" s="6" t="n"/>
-      <c r="D35" s="6" t="n"/>
+      <c r="D35" s="5" t="n"/>
+      <c r="E35" s="5" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="n"/>
-      <c r="B36" s="7" t="n"/>
+      <c r="A36" s="5" t="n"/>
+      <c r="B36" s="6" t="n"/>
       <c r="C36" s="6" t="n"/>
-      <c r="D36" s="6" t="n"/>
+      <c r="D36" s="5" t="n"/>
+      <c r="E36" s="5" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="n"/>
-      <c r="B37" s="7" t="n"/>
+      <c r="A37" s="5" t="n"/>
+      <c r="B37" s="6" t="n"/>
       <c r="C37" s="6" t="n"/>
-      <c r="D37" s="6" t="n"/>
+      <c r="D37" s="5" t="n"/>
+      <c r="E37" s="5" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="n"/>
-      <c r="B38" s="7" t="n"/>
+      <c r="A38" s="5" t="n"/>
+      <c r="B38" s="6" t="n"/>
       <c r="C38" s="6" t="n"/>
-      <c r="D38" s="6" t="n"/>
+      <c r="D38" s="5" t="n"/>
+      <c r="E38" s="5" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="n"/>
-      <c r="B39" s="7" t="n"/>
+      <c r="A39" s="5" t="n"/>
+      <c r="B39" s="6" t="n"/>
       <c r="C39" s="6" t="n"/>
-      <c r="D39" s="6" t="n"/>
+      <c r="D39" s="5" t="n"/>
+      <c r="E39" s="5" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="n"/>
-      <c r="B40" s="7" t="n"/>
+      <c r="A40" s="5" t="n"/>
+      <c r="B40" s="6" t="n"/>
       <c r="C40" s="6" t="n"/>
-      <c r="D40" s="6" t="n"/>
+      <c r="D40" s="5" t="n"/>
+      <c r="E40" s="5" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="n"/>
-      <c r="B41" s="7" t="n"/>
+      <c r="A41" s="5" t="n"/>
+      <c r="B41" s="6" t="n"/>
       <c r="C41" s="6" t="n"/>
-      <c r="D41" s="6" t="n"/>
+      <c r="D41" s="5" t="n"/>
+      <c r="E41" s="5" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="n"/>
-      <c r="B42" s="7" t="n"/>
+      <c r="A42" s="5" t="n"/>
+      <c r="B42" s="6" t="n"/>
       <c r="C42" s="6" t="n"/>
-      <c r="D42" s="6" t="n"/>
+      <c r="D42" s="5" t="n"/>
+      <c r="E42" s="5" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="n"/>
-      <c r="B43" s="7" t="n"/>
+      <c r="A43" s="5" t="n"/>
+      <c r="B43" s="6" t="n"/>
       <c r="C43" s="6" t="n"/>
-      <c r="D43" s="6" t="n"/>
+      <c r="D43" s="5" t="n"/>
+      <c r="E43" s="5" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="6" t="n"/>
-      <c r="B44" s="7" t="n"/>
+      <c r="A44" s="5" t="n"/>
+      <c r="B44" s="6" t="n"/>
       <c r="C44" s="6" t="n"/>
-      <c r="D44" s="6" t="n"/>
+      <c r="D44" s="5" t="n"/>
+      <c r="E44" s="5" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="6" t="n"/>
-      <c r="B45" s="7" t="n"/>
+      <c r="A45" s="5" t="n"/>
+      <c r="B45" s="6" t="n"/>
       <c r="C45" s="6" t="n"/>
-      <c r="D45" s="6" t="n"/>
+      <c r="D45" s="5" t="n"/>
+      <c r="E45" s="5" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="n"/>
-      <c r="B46" s="7" t="n"/>
+      <c r="A46" s="5" t="n"/>
+      <c r="B46" s="6" t="n"/>
       <c r="C46" s="6" t="n"/>
-      <c r="D46" s="6" t="n"/>
+      <c r="D46" s="5" t="n"/>
+      <c r="E46" s="5" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="6" t="n"/>
-      <c r="B47" s="7" t="n"/>
+      <c r="A47" s="5" t="n"/>
+      <c r="B47" s="6" t="n"/>
       <c r="C47" s="6" t="n"/>
-      <c r="D47" s="6" t="n"/>
+      <c r="D47" s="5" t="n"/>
+      <c r="E47" s="5" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="6" t="n"/>
-      <c r="B48" s="7" t="n"/>
+      <c r="A48" s="5" t="n"/>
+      <c r="B48" s="6" t="n"/>
       <c r="C48" s="6" t="n"/>
-      <c r="D48" s="6" t="n"/>
+      <c r="D48" s="5" t="n"/>
+      <c r="E48" s="5" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="6" t="n"/>
-      <c r="B49" s="7" t="n"/>
+      <c r="A49" s="5" t="n"/>
+      <c r="B49" s="6" t="n"/>
       <c r="C49" s="6" t="n"/>
-      <c r="D49" s="6" t="n"/>
+      <c r="D49" s="5" t="n"/>
+      <c r="E49" s="5" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="6" t="n"/>
-      <c r="B50" s="7" t="n"/>
+      <c r="A50" s="5" t="n"/>
+      <c r="B50" s="6" t="n"/>
       <c r="C50" s="6" t="n"/>
-      <c r="D50" s="6" t="n"/>
+      <c r="D50" s="5" t="n"/>
+      <c r="E50" s="5" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="6" t="n"/>
-      <c r="B51" s="7" t="n"/>
+      <c r="A51" s="5" t="n"/>
+      <c r="B51" s="6" t="n"/>
       <c r="C51" s="6" t="n"/>
-      <c r="D51" s="6" t="n"/>
+      <c r="D51" s="5" t="n"/>
+      <c r="E51" s="5" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="6" t="n"/>
-      <c r="B52" s="7" t="n"/>
+      <c r="A52" s="5" t="n"/>
+      <c r="B52" s="6" t="n"/>
       <c r="C52" s="6" t="n"/>
-      <c r="D52" s="6" t="n"/>
+      <c r="D52" s="5" t="n"/>
+      <c r="E52" s="5" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="6" t="n"/>
-      <c r="B53" s="7" t="n"/>
+      <c r="A53" s="5" t="n"/>
+      <c r="B53" s="6" t="n"/>
       <c r="C53" s="6" t="n"/>
-      <c r="D53" s="6" t="n"/>
+      <c r="D53" s="5" t="n"/>
+      <c r="E53" s="5" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="6" t="n"/>
-      <c r="B54" s="7" t="n"/>
+      <c r="A54" s="5" t="n"/>
+      <c r="B54" s="6" t="n"/>
       <c r="C54" s="6" t="n"/>
-      <c r="D54" s="6" t="n"/>
+      <c r="D54" s="5" t="n"/>
+      <c r="E54" s="5" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="6" t="n"/>
-      <c r="B55" s="7" t="n"/>
+      <c r="A55" s="5" t="n"/>
+      <c r="B55" s="6" t="n"/>
       <c r="C55" s="6" t="n"/>
-      <c r="D55" s="6" t="n"/>
+      <c r="D55" s="5" t="n"/>
+      <c r="E55" s="5" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="6" t="n"/>
-      <c r="B56" s="7" t="n"/>
+      <c r="A56" s="5" t="n"/>
+      <c r="B56" s="6" t="n"/>
       <c r="C56" s="6" t="n"/>
-      <c r="D56" s="6" t="n"/>
+      <c r="D56" s="5" t="n"/>
+      <c r="E56" s="5" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="6" t="n"/>
-      <c r="B57" s="7" t="n"/>
+      <c r="A57" s="5" t="n"/>
+      <c r="B57" s="6" t="n"/>
       <c r="C57" s="6" t="n"/>
-      <c r="D57" s="6" t="n"/>
+      <c r="D57" s="5" t="n"/>
+      <c r="E57" s="5" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="6" t="n"/>
-      <c r="B58" s="7" t="n"/>
+      <c r="A58" s="5" t="n"/>
+      <c r="B58" s="6" t="n"/>
       <c r="C58" s="6" t="n"/>
-      <c r="D58" s="6" t="n"/>
+      <c r="D58" s="5" t="n"/>
+      <c r="E58" s="5" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="6" t="n"/>
-      <c r="B59" s="7" t="n"/>
+      <c r="A59" s="5" t="n"/>
+      <c r="B59" s="6" t="n"/>
       <c r="C59" s="6" t="n"/>
-      <c r="D59" s="6" t="n"/>
+      <c r="D59" s="5" t="n"/>
+      <c r="E59" s="5" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="6" t="n"/>
-      <c r="B60" s="7" t="n"/>
+      <c r="A60" s="5" t="n"/>
+      <c r="B60" s="6" t="n"/>
       <c r="C60" s="6" t="n"/>
-      <c r="D60" s="6" t="n"/>
+      <c r="D60" s="5" t="n"/>
+      <c r="E60" s="5" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="6" t="n"/>
-      <c r="B61" s="7" t="n"/>
+      <c r="A61" s="5" t="n"/>
+      <c r="B61" s="6" t="n"/>
       <c r="C61" s="6" t="n"/>
-      <c r="D61" s="6" t="n"/>
+      <c r="D61" s="5" t="n"/>
+      <c r="E61" s="5" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="6" t="n"/>
-      <c r="B62" s="7" t="n"/>
+      <c r="A62" s="5" t="n"/>
+      <c r="B62" s="6" t="n"/>
       <c r="C62" s="6" t="n"/>
-      <c r="D62" s="6" t="n"/>
+      <c r="D62" s="5" t="n"/>
+      <c r="E62" s="5" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="6" t="n"/>
-      <c r="B63" s="7" t="n"/>
+      <c r="A63" s="5" t="n"/>
+      <c r="B63" s="6" t="n"/>
       <c r="C63" s="6" t="n"/>
-      <c r="D63" s="6" t="n"/>
+      <c r="D63" s="5" t="n"/>
+      <c r="E63" s="5" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="6" t="n"/>
-      <c r="B64" s="7" t="n"/>
+      <c r="A64" s="5" t="n"/>
+      <c r="B64" s="6" t="n"/>
       <c r="C64" s="6" t="n"/>
-      <c r="D64" s="6" t="n"/>
+      <c r="D64" s="5" t="n"/>
+      <c r="E64" s="5" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="6" t="n"/>
-      <c r="B65" s="7" t="n"/>
+      <c r="A65" s="5" t="n"/>
+      <c r="B65" s="6" t="n"/>
       <c r="C65" s="6" t="n"/>
-      <c r="D65" s="6" t="n"/>
+      <c r="D65" s="5" t="n"/>
+      <c r="E65" s="5" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="6" t="n"/>
-      <c r="B66" s="7" t="n"/>
+      <c r="A66" s="5" t="n"/>
+      <c r="B66" s="6" t="n"/>
       <c r="C66" s="6" t="n"/>
-      <c r="D66" s="6" t="n"/>
+      <c r="D66" s="5" t="n"/>
+      <c r="E66" s="5" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="6" t="n"/>
-      <c r="B67" s="7" t="n"/>
+      <c r="A67" s="5" t="n"/>
+      <c r="B67" s="6" t="n"/>
       <c r="C67" s="6" t="n"/>
-      <c r="D67" s="6" t="n"/>
+      <c r="D67" s="5" t="n"/>
+      <c r="E67" s="5" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="6" t="n"/>
-      <c r="B68" s="7" t="n"/>
+      <c r="A68" s="5" t="n"/>
+      <c r="B68" s="6" t="n"/>
       <c r="C68" s="6" t="n"/>
-      <c r="D68" s="6" t="n"/>
+      <c r="D68" s="5" t="n"/>
+      <c r="E68" s="5" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="6" t="n"/>
-      <c r="B69" s="7" t="n"/>
+      <c r="A69" s="5" t="n"/>
+      <c r="B69" s="6" t="n"/>
       <c r="C69" s="6" t="n"/>
-      <c r="D69" s="6" t="n"/>
+      <c r="D69" s="5" t="n"/>
+      <c r="E69" s="5" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="6" t="n"/>
-      <c r="B70" s="7" t="n"/>
+      <c r="A70" s="5" t="n"/>
+      <c r="B70" s="6" t="n"/>
       <c r="C70" s="6" t="n"/>
-      <c r="D70" s="6" t="n"/>
+      <c r="D70" s="5" t="n"/>
+      <c r="E70" s="5" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="6" t="n"/>
-      <c r="B71" s="7" t="n"/>
+      <c r="A71" s="5" t="n"/>
+      <c r="B71" s="6" t="n"/>
       <c r="C71" s="6" t="n"/>
-      <c r="D71" s="6" t="n"/>
+      <c r="D71" s="5" t="n"/>
+      <c r="E71" s="5" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="6" t="n"/>
-      <c r="B72" s="7" t="n"/>
+      <c r="A72" s="5" t="n"/>
+      <c r="B72" s="6" t="n"/>
       <c r="C72" s="6" t="n"/>
-      <c r="D72" s="6" t="n"/>
+      <c r="D72" s="5" t="n"/>
+      <c r="E72" s="5" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="6" t="n"/>
-      <c r="B73" s="7" t="n"/>
+      <c r="A73" s="5" t="n"/>
+      <c r="B73" s="6" t="n"/>
       <c r="C73" s="6" t="n"/>
-      <c r="D73" s="6" t="n"/>
+      <c r="D73" s="5" t="n"/>
+      <c r="E73" s="5" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="6" t="n"/>
-      <c r="B74" s="7" t="n"/>
+      <c r="A74" s="5" t="n"/>
+      <c r="B74" s="6" t="n"/>
       <c r="C74" s="6" t="n"/>
-      <c r="D74" s="6" t="n"/>
+      <c r="D74" s="5" t="n"/>
+      <c r="E74" s="5" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="6" t="n"/>
-      <c r="B75" s="7" t="n"/>
+      <c r="A75" s="5" t="n"/>
+      <c r="B75" s="6" t="n"/>
       <c r="C75" s="6" t="n"/>
-      <c r="D75" s="6" t="n"/>
+      <c r="D75" s="5" t="n"/>
+      <c r="E75" s="5" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="6" t="n"/>
-      <c r="B76" s="7" t="n"/>
+      <c r="A76" s="5" t="n"/>
+      <c r="B76" s="6" t="n"/>
       <c r="C76" s="6" t="n"/>
-      <c r="D76" s="6" t="n"/>
+      <c r="D76" s="5" t="n"/>
+      <c r="E76" s="5" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="6" t="n"/>
-      <c r="B77" s="7" t="n"/>
+      <c r="A77" s="5" t="n"/>
+      <c r="B77" s="6" t="n"/>
       <c r="C77" s="6" t="n"/>
-      <c r="D77" s="6" t="n"/>
+      <c r="D77" s="5" t="n"/>
+      <c r="E77" s="5" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="6" t="n"/>
-      <c r="B78" s="7" t="n"/>
+      <c r="A78" s="5" t="n"/>
+      <c r="B78" s="6" t="n"/>
       <c r="C78" s="6" t="n"/>
-      <c r="D78" s="6" t="n"/>
+      <c r="D78" s="5" t="n"/>
+      <c r="E78" s="5" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="6" t="n"/>
-      <c r="B79" s="7" t="n"/>
+      <c r="A79" s="5" t="n"/>
+      <c r="B79" s="6" t="n"/>
       <c r="C79" s="6" t="n"/>
-      <c r="D79" s="6" t="n"/>
+      <c r="D79" s="5" t="n"/>
+      <c r="E79" s="5" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="6" t="n"/>
-      <c r="B80" s="7" t="n"/>
+      <c r="A80" s="5" t="n"/>
+      <c r="B80" s="6" t="n"/>
       <c r="C80" s="6" t="n"/>
-      <c r="D80" s="6" t="n"/>
+      <c r="D80" s="5" t="n"/>
+      <c r="E80" s="5" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="6" t="n"/>
-      <c r="B81" s="7" t="n"/>
+      <c r="A81" s="5" t="n"/>
+      <c r="B81" s="6" t="n"/>
       <c r="C81" s="6" t="n"/>
-      <c r="D81" s="6" t="n"/>
+      <c r="D81" s="5" t="n"/>
+      <c r="E81" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C7:C81" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Position" prompt="Pick one or type your own." type="list" errorStyle="information">
+    <dataValidation sqref="D7:D81" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Position" prompt="Pick one or type your own." type="list">
       <formula1>"Server,Bartender,Host,Busser,Line Cook,Prep Cook,Sous Chef,Dishwasher,Manager,Sommelier,Event Staff"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>